<commit_message>
deleted the "URL ID" row
</commit_message>
<xml_diff>
--- a/Dataset - Daily Caffeine Consumption and Lecture Concentration.xlsx
+++ b/Dataset - Daily Caffeine Consumption and Lecture Concentration.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucaswang/Desktop/STA304/Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD4A9FDB-EF82-FE4C-91AC-201E3AA328AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FB5663B-364D-0D46-9A98-FD359FF7BD79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12580" yWindow="3140" windowWidth="26740" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7460" yWindow="3140" windowWidth="26740" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Form Responses 1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
   <si>
     <t>studentID</t>
   </si>
@@ -177,9 +177,6 @@
   </si>
   <si>
     <t>LaTexSupremacy11</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/e/1FAIpQLSeA6EAI8MAVNOU3EEXFpD7ZBhiIcfiocILYZzYOcAoAn8vuJQ/viewform</t>
   </si>
   <si>
     <t>wwUs</t>
@@ -267,7 +264,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -280,12 +277,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Roboto"/>
     </font>
   </fonts>
   <fills count="2">
@@ -308,12 +299,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -429,7 +417,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:K66" headerRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:K65" headerRowDxfId="1">
   <tableColumns count="11">
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="studentID"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Section"/>
@@ -650,7 +638,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:K66"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
@@ -667,39 +655,39 @@
     <col min="12" max="17" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="5" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="1:11" s="4" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -1874,7 +1862,7 @@
         <v>4</v>
       </c>
       <c r="G34" s="1">
-        <f t="shared" ref="G34:G65" si="1">SUM(C34, D34, E34, F34)</f>
+        <f t="shared" ref="G34:G64" si="1">SUM(C34, D34, E34, F34)</f>
         <v>12</v>
       </c>
       <c r="H34" s="1">
@@ -2395,14 +2383,14 @@
       </c>
     </row>
     <row r="49" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A49" s="2" t="s">
+      <c r="A49" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B49" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C49" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D49" s="1">
         <v>0</v>
@@ -2415,19 +2403,19 @@
       </c>
       <c r="G49" s="1">
         <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="H49" s="1">
+        <v>6</v>
+      </c>
+      <c r="I49" s="1">
+        <v>7</v>
+      </c>
+      <c r="J49" s="1">
         <v>3</v>
       </c>
-      <c r="H49" s="1">
-        <v>5</v>
-      </c>
-      <c r="I49" s="1">
-        <v>9</v>
-      </c>
-      <c r="J49" s="1">
-        <v>5</v>
-      </c>
       <c r="K49" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2435,10 +2423,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D50" s="1">
         <v>0</v>
@@ -2451,19 +2439,19 @@
       </c>
       <c r="G50" s="1">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H50" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I50" s="1">
         <v>7</v>
       </c>
       <c r="J50" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K50" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2471,65 +2459,63 @@
         <v>50</v>
       </c>
       <c r="B51" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C51" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D51" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E51" s="1">
         <v>0</v>
       </c>
       <c r="F51" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G51" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H51" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I51" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J51" s="1">
         <v>5</v>
       </c>
       <c r="K51" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B52" s="1">
-        <v>2</v>
-      </c>
+      <c r="B52" s="1"/>
       <c r="C52" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D52" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E52" s="1">
         <v>0</v>
       </c>
       <c r="F52" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G52" s="1">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H52" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I52" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J52" s="1">
         <v>5</v>
@@ -2542,34 +2528,36 @@
       <c r="A53" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B53" s="1"/>
+      <c r="B53" s="1">
+        <v>2</v>
+      </c>
       <c r="C53" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D53" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E53" s="1">
         <v>0</v>
       </c>
       <c r="F53" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G53" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H53" s="1">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I53" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J53" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K53" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2580,32 +2568,32 @@
         <v>2</v>
       </c>
       <c r="C54" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D54" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E54" s="1">
         <v>0</v>
       </c>
       <c r="F54" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G54" s="1">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H54" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I54" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J54" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K54" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2613,10 +2601,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D55" s="1">
         <v>0</v>
@@ -2629,19 +2617,19 @@
       </c>
       <c r="G55" s="1">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H55" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I55" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J55" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K55" s="1">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="56" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2649,23 +2637,23 @@
         <v>55</v>
       </c>
       <c r="B56" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C56" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D56" s="1">
         <v>0</v>
       </c>
       <c r="E56" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F56" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G56" s="1">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H56" s="1">
         <v>6</v>
@@ -2674,10 +2662,10 @@
         <v>8</v>
       </c>
       <c r="J56" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K56" s="1">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="57" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2685,7 +2673,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C57" s="1">
         <v>0</v>
@@ -2694,26 +2682,26 @@
         <v>0</v>
       </c>
       <c r="E57" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F57" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G57" s="1">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H57" s="1">
         <v>6</v>
       </c>
       <c r="I57" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J57" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K57" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2721,10 +2709,10 @@
         <v>57</v>
       </c>
       <c r="B58" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C58" s="1">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="D58" s="1">
         <v>0</v>
@@ -2737,10 +2725,10 @@
       </c>
       <c r="G58" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="H58" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I58" s="1">
         <v>6</v>
@@ -2749,7 +2737,7 @@
         <v>7</v>
       </c>
       <c r="K58" s="1">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2757,35 +2745,32 @@
         <v>58</v>
       </c>
       <c r="B59" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C59" s="1">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="D59" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E59" s="1">
         <v>0</v>
       </c>
-      <c r="F59" s="1">
-        <v>0</v>
-      </c>
-      <c r="G59" s="1">
+      <c r="G59">
         <f t="shared" si="1"/>
-        <v>1.9</v>
+        <v>3</v>
       </c>
       <c r="H59" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I59" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J59" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K59" s="1">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2796,29 +2781,32 @@
         <v>1</v>
       </c>
       <c r="C60" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D60" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E60" s="1">
         <v>0</v>
       </c>
-      <c r="G60">
+      <c r="F60" s="1">
+        <v>0</v>
+      </c>
+      <c r="G60" s="1">
         <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H60" s="1">
+        <v>9</v>
+      </c>
+      <c r="I60" s="1">
+        <v>6</v>
+      </c>
+      <c r="J60" s="1">
         <v>3</v>
       </c>
-      <c r="H60" s="1">
-        <v>1</v>
-      </c>
-      <c r="I60" s="1">
-        <v>9</v>
-      </c>
-      <c r="J60" s="1">
-        <v>9</v>
-      </c>
       <c r="K60" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="61" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2826,10 +2814,10 @@
         <v>60</v>
       </c>
       <c r="B61" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C61" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D61" s="1">
         <v>0</v>
@@ -2842,19 +2830,19 @@
       </c>
       <c r="G61" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H61" s="1">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I61" s="1">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="J61" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K61" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2865,7 +2853,7 @@
         <v>2</v>
       </c>
       <c r="C62" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D62" s="1">
         <v>0</v>
@@ -2878,19 +2866,19 @@
       </c>
       <c r="G62" s="1">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H62" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I62" s="1">
-        <v>7.5</v>
+        <v>11</v>
       </c>
       <c r="J62" s="1">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="K62" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="63" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2898,35 +2886,35 @@
         <v>62</v>
       </c>
       <c r="B63" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C63" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D63" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E63" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F63" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G63" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H63" s="1">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I63" s="1">
-        <v>11</v>
+        <v>6.5</v>
       </c>
       <c r="J63" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K63" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="64" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2934,35 +2922,35 @@
         <v>63</v>
       </c>
       <c r="B64" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C64" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D64" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E64" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F64" s="1">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G64" s="1">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H64" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I64" s="1">
-        <v>6.5</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="J64" s="1">
         <v>6</v>
       </c>
       <c r="K64" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="65" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2970,81 +2958,42 @@
         <v>64</v>
       </c>
       <c r="B65" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C65" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D65" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E65" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F65" s="1">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G65" s="1">
-        <f t="shared" si="1"/>
-        <v>10</v>
+        <f t="shared" ref="G65" si="2">SUM(C65, D65, E65, F65)</f>
+        <v>9</v>
       </c>
       <c r="H65" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I65" s="1">
-        <v>8.1999999999999993</v>
+        <v>6</v>
       </c>
       <c r="J65" s="1">
         <v>6</v>
       </c>
       <c r="K65" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A66" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B66" s="1">
-        <v>1</v>
-      </c>
-      <c r="C66" s="1">
-        <v>2</v>
-      </c>
-      <c r="D66" s="1">
-        <v>2</v>
-      </c>
-      <c r="E66" s="1">
-        <v>3</v>
-      </c>
-      <c r="F66" s="1">
-        <v>2</v>
-      </c>
-      <c r="G66" s="1">
-        <f t="shared" ref="G66:G97" si="2">SUM(C66, D66, E66, F66)</f>
-        <v>9</v>
-      </c>
-      <c r="H66" s="1">
-        <v>8</v>
-      </c>
-      <c r="I66" s="1">
-        <v>6</v>
-      </c>
-      <c r="J66" s="1">
-        <v>6</v>
-      </c>
-      <c r="K66" s="1">
         <v>4</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A49" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>